<commit_message>
Record the manual audit: 132 targeted cells, 0 errors
The five audit sheets were checked by hand against the PDFs (2026-10-02):
all cells correct. Sheets filled in, audit_result_<prov>.md written.
02_validate.py --score reports a targeted sheet by selection reason and no
longer prints a random-sample error bound for it. README, the October audit
report and the Torino pilot report now describe the targeted manual audit
instead of the 200-cell random one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011mvLWFfLFbnKm7v6S9L2EZ
</commit_message>
<xml_diff>
--- a/output/audit_alessandria.xlsx
+++ b/output/audit_alessandria.xlsx
@@ -535,9 +535,17 @@
           <t>4</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -576,9 +584,17 @@
           <t>5</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -617,9 +633,17 @@
           <t>3</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -658,9 +682,17 @@
           <t>1.682,46</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -699,9 +731,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -740,9 +780,17 @@
           <t>7,85</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -781,9 +829,17 @@
           <t>454</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -822,9 +878,17 @@
           <t>3.701,14</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -863,9 +927,17 @@
           <t>387,59</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -904,9 +976,17 @@
           <t>534,08</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -945,9 +1025,17 @@
           <t>1.809,50</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -986,9 +1074,17 @@
           <t>609,53</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1027,9 +1123,17 @@
           <t>1.098,60</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1068,9 +1172,17 @@
           <t>1.558,09</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1109,9 +1221,17 @@
           <t>519,79</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1150,9 +1270,17 @@
           <t>23.252,99</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1191,9 +1319,17 @@
           <t>26</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>controllo: OCR e lettura visiva concordi</t>
@@ -1232,9 +1368,17 @@
           <t>52,90</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1273,9 +1417,17 @@
           <t>818,73</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1314,9 +1466,17 @@
           <t>784,14</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1355,9 +1515,17 @@
           <t>3.154,79</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1396,9 +1564,17 @@
           <t>3.234,40</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1437,9 +1613,17 @@
           <t>1.900,30</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1478,9 +1662,17 @@
           <t>2.155,62</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>controllo manuale sul PDF, 2026-10-02</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>riletta su zoom / ricostruita da somma di riga</t>
@@ -1516,9 +1708,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1554,9 +1744,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1592,9 +1780,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>

</xml_diff>